<commit_message>
Update conftest for CI headless mode
</commit_message>
<xml_diff>
--- a/report/test_results_order.xlsx
+++ b/report/test_results_order.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Order Test Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,16 +413,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -455,6 +447,66 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Unnamed: 6</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Unnamed: 7</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Unnamed: 8</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Unnamed: 9</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Unnamed: 10</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Province</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Actual Error</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -487,6 +539,18 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -519,6 +583,18 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -551,6 +627,18 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -583,6 +671,18 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -600,6 +700,7 @@
           <t>SWE CROSS SWEATPANTS - GRAY</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>0912345678</t>
@@ -635,6 +736,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -657,6 +765,7 @@
           <t>bình</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>namanh@gmail.com</t>
@@ -687,6 +796,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -744,6 +860,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -776,6 +899,7 @@
           <t>chiecgiuong@gmail.com</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
@@ -796,6 +920,13 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -853,6 +984,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -870,6 +1008,7 @@
           <t>SWE CROSS SWEATPANTS - GRAY</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>0912345678</t>
@@ -905,6 +1044,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -927,6 +1073,7 @@
           <t>bình</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>namanh@gmail.com</t>
@@ -957,6 +1104,13 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1014,6 +1168,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1046,6 +1207,7 @@
           <t>chiecgiuong@gmail.com</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
@@ -1066,6 +1228,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1123,6 +1292,13 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1140,6 +1316,7 @@
           <t>SWE CROSS SWEATPANTS - GRAY</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>0912345678</t>
@@ -1175,6 +1352,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1197,6 +1381,7 @@
           <t>bình</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>namanh@gmail.com</t>
@@ -1227,6 +1412,13 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1284,6 +1476,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1316,6 +1515,7 @@
           <t>chiecgiuong@gmail.com</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
@@ -1336,6 +1536,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1393,6 +1600,13 @@
           <t>FAIL</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1410,6 +1624,7 @@
           <t>SWE CROSS SWEATPANTS - GRAY</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>0912345678</t>
@@ -1445,6 +1660,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1467,6 +1689,7 @@
           <t>bình</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>namanh@gmail.com</t>
@@ -1497,6 +1720,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1554,6 +1784,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1586,6 +1823,7 @@
           <t>chiecgiuong@gmail.com</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
@@ -1606,6 +1844,13 @@
           <t>PASS</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1661,6 +1906,1174 @@
       <c r="K25" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-08 09:15:53</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>checkout_name_SWE CROSS SW</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>SWE CROSS SWEATPANTS - GRAY</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>912345678</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>namanh@gmail.com</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Vui lòng nhập họ tên</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-08 09:16:30</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>checkout_phone_SWE SPIKE BO</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>SWE SPIKE BOXY TEE - WHITE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>bình</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>namanh@gmail.com</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Message: 
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x7ff6d99329c5+2ed785]
+	chromedriver!GetHandleVerifier [0x7ff6d965a0d0+14e90]
+	chromedriver!(No symbol) [0x7ff6d93bdb2d]
+	chromedriver!(No symbol) [0x7ff6d9416b9e]
+	chromedriver!(No symbol) [0x7ff6d9416eac]
+	chromedriver!(No symbol) [0x7ff6d9466fe7]
+	chromedriver!(No symbol) [0x7ff6d9463b9b]
+	chromedriver!(No symbol) [0x7ff6d9409298]
+	chromedriver!(No symbol) [0x7ff6d940a183]
+	chromedriver!GetHandleVerifier [0x7ff6d995de0d+318bcd]
+	chromedriver!GetHandleVerifier [0x7ff6d9958588+313348]
+	chromedriver!GetHandleVerifier [0x7ff6d9979d7a+334b3a]
+	chromedriver!GetHandleVerifier [0x7ff6d9676785+31545]
+	chromedriver!GetHandleVerifier [0x7ff6d967facc+3a88c]
+	chromedriver!GetHandleVerifier [0x7ff6d9663634+1e3f4]
+	chromedriver!GetHandleVerifier [0x7ff6d96637e6+1e5a6]
+	chromedriver!GetHandleVerifier [0x7ff6d9647e37+2bf7]
+	KERNEL32!BaseThreadInitThunk [0x7ff9e8ef7374+14]
+	ntdll!RtlUserThreadStart [0x7ff9eae5cc91+21]
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-08 09:16:49</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>checkout_email_SWE PIPELINE</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>SWE PIPELINE JEANS - RETRO BLUE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>an</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>97736452</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>binhyennhungphutgiay</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Message: 
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x7ff6d99329c5+2ed785]
+	chromedriver!GetHandleVerifier [0x7ff6d965a0d0+14e90]
+	chromedriver!(No symbol) [0x7ff6d93bdb2d]
+	chromedriver!(No symbol) [0x7ff6d9416b9e]
+	chromedriver!(No symbol) [0x7ff6d9416eac]
+	chromedriver!(No symbol) [0x7ff6d9466fe7]
+	chromedriver!(No symbol) [0x7ff6d9463b9b]
+	chromedriver!(No symbol) [0x7ff6d9409298]
+	chromedriver!(No symbol) [0x7ff6d940a183]
+	chromedriver!GetHandleVerifier [0x7ff6d995de0d+318bcd]
+	chromedriver!GetHandleVerifier [0x7ff6d9958588+313348]
+	chromedriver!GetHandleVerifier [0x7ff6d9979d7a+334b3a]
+	chromedriver!GetHandleVerifier [0x7ff6d9676785+31545]
+	chromedriver!GetHandleVerifier [0x7ff6d967facc+3a88c]
+	chromedriver!GetHandleVerifier [0x7ff6d9663634+1e3f4]
+	chromedriver!GetHandleVerifier [0x7ff6d96637e6+1e5a6]
+	chromedriver!GetHandleVerifier [0x7ff6d9647e37+2bf7]
+	KERNEL32!BaseThreadInitThunk [0x7ff9e8ef7374+14]
+	ntdll!RtlUserThreadStart [0x7ff9eae5cc91+21]
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-08 09:19:18</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>checkout_name_SWE CROSS SW</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>SWE CROSS SWEATPANTS - GRAY</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>912345678</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>namanh@gmail.com</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Vui lòng nhập họ tên</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-08 09:20:02</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>checkout_phone_SWE SPIKE BO</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>SWE SPIKE BOXY TEE - WHITE</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>bình</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>namanh@gmail.com</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Message: timeout: Timed out receiving message from renderer: 39.820
+  (Session info: chrome=146.0.7680.178)
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x7ff7ef3e29c5+2ed785]
+	chromedriver!GetHandleVerifier [0x7ff7ef10a0d0+14e90]
+	chromedriver!(No symbol) [0x7ff7eee6db2d]
+	chromedriver!(No symbol) [0x7ff7eee5a409]
+	chromedriver!(No symbol) [0x7ff7eee5a0f1]
+	chromedriver!(No symbol) [0x7ff7eee57d3b]
+	chromedriver!(No symbol) [0x7ff7eee5865f]
+	chromedriver!(No symbol) [0x7ff7eee67eca]
+	chromedriver!(No symbol) [0x7ff7eee7edf7]
+	chromedriver!(No symbol) [0x7ff7eee8654a]
+	chromedriver!(No symbol) [0x7ff7eee58e21]
+	chromedriver!(No symbol) [0x7ff7eee7eb21]
+	chromedriver!(No symbol) [0x7ff7eef13f14]
+	chromedriver!(No symbol) [0x7ff7eeeb9298]
+	chromedriver!(No symbol) [0x7ff7eeeba183]
+	chromedriver!GetHandleVerifier [0x7ff7ef40de0d+318bcd]
+	chromedriver!GetHandleVerifier [0x7ff7ef408588+313348]
+	chromedriver!GetHandleVerifier [0x7ff7ef429d7a+334b3a]
+	chromedriver!GetHandleVerifier [0x7ff7ef126785+31545]
+	chromedriver!GetHandleVerifier [0x7ff7ef12facc+3a88c]
+	chromedriver!GetHandleVerifier [0x7ff7ef113634+1e3f4]
+	chromedriver!GetHandleVerifier [0x7ff7ef1137e6+1e5a6]
+	chromedriver!GetHandleVerifier [0x7ff7ef0f7e37+2bf7]
+	KERNEL32!BaseThreadInitThunk [0x7ff9e8ef7374+14]
+	ntdll!RtlUserThreadStart [0x7ff9eae5cc91+21]
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-08 09:20:43</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>checkout_email_SWE PIPELINE</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>SWE PIPELINE JEANS - RETRO BLUE</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>an</t>
+        </is>
+      </c>
+      <c r="M31" t="n">
+        <v>97736452</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>binhyennhungphutgiay</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Message: 
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x7ff7ef3e29c5+2ed785]
+	chromedriver!GetHandleVerifier [0x7ff7ef10a0d0+14e90]
+	chromedriver!(No symbol) [0x7ff7eee6db2d]
+	chromedriver!(No symbol) [0x7ff7eeec6b9e]
+	chromedriver!(No symbol) [0x7ff7eeec6eac]
+	chromedriver!(No symbol) [0x7ff7eef16fe7]
+	chromedriver!(No symbol) [0x7ff7eef13b9b]
+	chromedriver!(No symbol) [0x7ff7eeeb9298]
+	chromedriver!(No symbol) [0x7ff7eeeba183]
+	chromedriver!GetHandleVerifier [0x7ff7ef40de0d+318bcd]
+	chromedriver!GetHandleVerifier [0x7ff7ef408588+313348]
+	chromedriver!GetHandleVerifier [0x7ff7ef429d7a+334b3a]
+	chromedriver!GetHandleVerifier [0x7ff7ef126785+31545]
+	chromedriver!GetHandleVerifier [0x7ff7ef12facc+3a88c]
+	chromedriver!GetHandleVerifier [0x7ff7ef113634+1e3f4]
+	chromedriver!GetHandleVerifier [0x7ff7ef1137e6+1e5a6]
+	chromedriver!GetHandleVerifier [0x7ff7ef0f7e37+2bf7]
+	KERNEL32!BaseThreadInitThunk [0x7ff9e8ef7374+14]
+	ntdll!RtlUserThreadStart [0x7ff9eae5cc91+21]
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-08 09:21:32</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>checkout_province_SWE SCRIPT J</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>SWE SCRIPT JACKET - BEIGE</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>an</t>
+        </is>
+      </c>
+      <c r="M32" t="n">
+        <v>97736453</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>chiecgiuong@gmail.com</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>province</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Vui lòng chọn tỉnh thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-08 09:22:16</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>checkout_phone_SWE LIFE TEE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>SWE LIFE TEE - BLACK</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>mai</t>
+        </is>
+      </c>
+      <c r="M33" t="n">
+        <v>97523746</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>test@gmail.com</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Message: timeout: Timed out receiving message from renderer: 38.386
+  (Session info: chrome=146.0.7680.178)
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x7ff7ef3e29c5+2ed785]
+	chromedriver!GetHandleVerifier [0x7ff7ef10a0d0+14e90]
+	chromedriver!(No symbol) [0x7ff7eee6db2d]
+	chromedriver!(No symbol) [0x7ff7eee5a409]
+	chromedriver!(No symbol) [0x7ff7eee5a0f1]
+	chromedriver!(No symbol) [0x7ff7eee57d3b]
+	chromedriver!(No symbol) [0x7ff7eee5865f]
+	chromedriver!(No symbol) [0x7ff7eee67eca]
+	chromedriver!(No symbol) [0x7ff7eee7edf7]
+	chromedriver!(No symbol) [0x7ff7eee8654a]
+	chromedriver!(No symbol) [0x7ff7eee58e21]
+	chromedriver!(No symbol) [0x7ff7eee7eb21]
+	chromedriver!(No symbol) [0x7ff7eef13f14]
+	chromedriver!(No symbol) [0x7ff7eeeb9298]
+	chromedriver!(No symbol) [0x7ff7eeeba183]
+	chromedriver!GetHandleVerifier [0x7ff7ef40de0d+318bcd]
+	chromedriver!GetHandleVerifier [0x7ff7ef408588+313348]
+	chromedriver!GetHandleVerifier [0x7ff7ef429d7a+334b3a]
+	chromedriver!GetHandleVerifier [0x7ff7ef126785+31545]
+	chromedriver!GetHandleVerifier [0x7ff7ef12facc+3a88c]
+	chromedriver!GetHandleVerifier [0x7ff7ef113634+1e3f4]
+	chromedriver!GetHandleVerifier [0x7ff7ef1137e6+1e5a6]
+	chromedriver!GetHandleVerifier [0x7ff7ef0f7e37+2bf7]
+	KERNEL32!BaseThreadInitThunk [0x7ff9e8ef7374+14]
+	ntdll!RtlUserThreadStart [0x7ff9eae5cc91+21]
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-05-08 09:34:04</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>checkout_name_SWE CROSS SW</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SWE CROSS SWEATPANTS - GRAY</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="n">
+        <v>912345678</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>namanh@gmail.com</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Vui lòng nhập họ tên</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-05-08 09:34:35</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>checkout_phone_SWE SPIKE BO</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>SWE SPIKE BOXY TEE - WHITE</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>bình</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>namanh@gmail.com</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Message: 
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x7ff74e8d29c5+2ed785]
+	chromedriver!GetHandleVerifier [0x7ff74e5fa0d0+14e90]
+	chromedriver!(No symbol) [0x7ff74e35db2d]
+	chromedriver!(No symbol) [0x7ff74e3b6b9e]
+	chromedriver!(No symbol) [0x7ff74e3b6eac]
+	chromedriver!(No symbol) [0x7ff74e406fe7]
+	chromedriver!(No symbol) [0x7ff74e403b9b]
+	chromedriver!(No symbol) [0x7ff74e3a9298]
+	chromedriver!(No symbol) [0x7ff74e3aa183]
+	chromedriver!GetHandleVerifier [0x7ff74e8fde0d+318bcd]
+	chromedriver!GetHandleVerifier [0x7ff74e8f8588+313348]
+	chromedriver!GetHandleVerifier [0x7ff74e919d7a+334b3a]
+	chromedriver!GetHandleVerifier [0x7ff74e616785+31545]
+	chromedriver!GetHandleVerifier [0x7ff74e61facc+3a88c]
+	chromedriver!GetHandleVerifier [0x7ff74e603634+1e3f4]
+	chromedriver!GetHandleVerifier [0x7ff74e6037e6+1e5a6]
+	chromedriver!GetHandleVerifier [0x7ff74e5e7e37+2bf7]
+	KERNEL32!BaseThreadInitThunk [0x7ff9e8ef7374+14]
+	ntdll!RtlUserThreadStart [0x7ff9eae5cc91+21]
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-08 09:34:41</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>checkout_email_SWE PIPELINE</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>SWE PIPELINE JEANS - RETRO BLUE</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>an</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>97736452</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>binhyennhungphutgiay</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05-08 21:35:14</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>checkout_name_SWE CROSS SW</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SWE CROSS SWEATPANTS - GRAY</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="n">
+        <v>912345678</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>namanh@gmail.com</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Vui lòng nhập họ tên</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-05-08 21:35:43</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>checkout_phone_SWE SPIKE BO</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>SWE SPIKE BOXY TEE - WHITE</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>bình</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>namanh@gmail.com</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Message: 
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x7ff7c12129c5+2ed785]
+	chromedriver!GetHandleVerifier [0x7ff7c0f3a0d0+14e90]
+	chromedriver!(No symbol) [0x7ff7c0c9db2d]
+	chromedriver!(No symbol) [0x7ff7c0cf6b9e]
+	chromedriver!(No symbol) [0x7ff7c0cf6eac]
+	chromedriver!(No symbol) [0x7ff7c0d46fe7]
+	chromedriver!(No symbol) [0x7ff7c0d43b9b]
+	chromedriver!(No symbol) [0x7ff7c0ce9298]
+	chromedriver!(No symbol) [0x7ff7c0cea183]
+	chromedriver!GetHandleVerifier [0x7ff7c123de0d+318bcd]
+	chromedriver!GetHandleVerifier [0x7ff7c1238588+313348]
+	chromedriver!GetHandleVerifier [0x7ff7c1259d7a+334b3a]
+	chromedriver!GetHandleVerifier [0x7ff7c0f56785+31545]
+	chromedriver!GetHandleVerifier [0x7ff7c0f5facc+3a88c]
+	chromedriver!GetHandleVerifier [0x7ff7c0f43634+1e3f4]
+	chromedriver!GetHandleVerifier [0x7ff7c0f437e6+1e5a6]
+	chromedriver!GetHandleVerifier [0x7ff7c0f27e37+2bf7]
+	KERNEL32!BaseThreadInitThunk [0x7ff9e8ef7374+14]
+	ntdll!RtlUserThreadStart [0x7ff9eae5cc91+21]
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-05-08 21:36:11</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>checkout_email_SWE PIPELINE</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SWE PIPELINE JEANS - RETRO BLUE</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>an</t>
+        </is>
+      </c>
+      <c r="M39" t="n">
+        <v>97736452</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>binhyennhungphutgiay</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Message: 
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x7ff7c12129c5+2ed785]
+	chromedriver!GetHandleVerifier [0x7ff7c0f3a0d0+14e90]
+	chromedriver!(No symbol) [0x7ff7c0c9db2d]
+	chromedriver!(No symbol) [0x7ff7c0cf6b9e]
+	chromedriver!(No symbol) [0x7ff7c0cf6eac]
+	chromedriver!(No symbol) [0x7ff7c0d46fe7]
+	chromedriver!(No symbol) [0x7ff7c0d43b9b]
+	chromedriver!(No symbol) [0x7ff7c0ce9298]
+	chromedriver!(No symbol) [0x7ff7c0cea183]
+	chromedriver!GetHandleVerifier [0x7ff7c123de0d+318bcd]
+	chromedriver!GetHandleVerifier [0x7ff7c1238588+313348]
+	chromedriver!GetHandleVerifier [0x7ff7c1259d7a+334b3a]
+	chromedriver!GetHandleVerifier [0x7ff7c0f56785+31545]
+	chromedriver!GetHandleVerifier [0x7ff7c0f5facc+3a88c]
+	chromedriver!GetHandleVerifier [0x7ff7c0f43634+1e3f4]
+	chromedriver!GetHandleVerifier [0x7ff7c0f437e6+1e5a6]
+	chromedriver!GetHandleVerifier [0x7ff7c0f27e37+2bf7]
+	KERNEL32!BaseThreadInitThunk [0x7ff9e8ef7374+14]
+	ntdll!RtlUserThreadStart [0x7ff9eae5cc91+21]
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-05-08 21:36:33</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>checkout_province_SWE SCRIPT J</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>SWE SCRIPT JACKET - BEIGE</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>an</t>
+        </is>
+      </c>
+      <c r="M40" t="n">
+        <v>97736453</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>chiecgiuong@gmail.com</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>province</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Vui lòng chọn tỉnh thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-05-08 21:37:01</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>checkout_phone_SWE LIFE TEE</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>SWE LIFE TEE - BLACK</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>mai</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>097523746</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>test@gmail.com</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Thị trấn Xuân Mai, Huyện Chương Mỹ, Hà Nội</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Message: 
+Stacktrace:
+	chromedriver!GetHandleVerifier [0x7ff7c12129c5+2ed785]
+	chromedriver!GetHandleVerifier [0x7ff7c0f3a0d0+14e90]
+	chromedriver!(No symbol) [0x7ff7c0c9db2d]
+	chromedriver!(No symbol) [0x7ff7c0cf6b9e]
+	chromedriver!(No symbol) [0x7ff7c0cf6eac]
+	chromedriver!(No symbol) [0x7ff7c0d46fe7]
+	chromedriver!(No symbol) [0x7ff7c0d43b9b]
+	chromedriver!(No symbol) [0x7ff7c0ce9298]
+	chromedriver!(No symbol) [0x7ff7c0cea183]
+	chromedriver!GetHandleVerifier [0x7ff7c123de0d+318bcd]
+	chromedriver!GetHandleVerifier [0x7ff7c1238588+313348]
+	chromedriver!GetHandleVerifier [0x7ff7c1259d7a+334b3a]
+	chromedriver!GetHandleVerifier [0x7ff7c0f56785+31545]
+	chromedriver!GetHandleVerifier [0x7ff7c0f5facc+3a88c]
+	chromedriver!GetHandleVerifier [0x7ff7c0f43634+1e3f4]
+	chromedriver!GetHandleVerifier [0x7ff7c0f437e6+1e5a6]
+	chromedriver!GetHandleVerifier [0x7ff7c0f27e37+2bf7]
+	KERNEL32!BaseThreadInitThunk [0x7ff9e8ef7374+14]
+	ntdll!RtlUserThreadStart [0x7ff9eae5cc91+21]
+</t>
         </is>
       </c>
     </row>

</xml_diff>